<commit_message>
Completa Puntos/Ranking FIFA de las 48 selecciones (0 imputados)
- Carga Puntos y Ranking FIFA de las 11 selecciones que faltaban (antes imputadas con mediana de confederacion - 40).
- Ranking: posiciones exactas del 19-nov-2025 (fuente: ranking del sorteo del Mundial; validado contra las 5 ya presentes, coinciden).
- Puntos: reconstruidos del rank exacto via recta rank->puntos del propio Excel (pendiente -3.34 pts/rank, RMSE cola 2.0; validado vs Arabia Saudita real ±4). Son estimaciones ±~5 pts, no los decimales literales.
- Efecto: 0 imputados (antes 11); mejora log-loss CV (logit 1.004->0.922, gbm 1.344->1.207) y recalibra la fuerza de esos equipos y sus rivales.
- Docs: documenta el metodo y deja como pendiente opcional reemplazar por decimales exactos de FIFA.com.
</commit_message>
<xml_diff>
--- a/Mundial_2026_fuente_datos.xlsx
+++ b/Mundial_2026_fuente_datos.xlsx
@@ -986,8 +986,12 @@
           <t>CAF</t>
         </is>
       </c>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="12" t="n"/>
+      <c r="G4" s="10" t="n">
+        <v>61</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>1427.3</v>
+      </c>
       <c r="I4" s="10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1170,8 +1174,12 @@
           <t>UEFA</t>
         </is>
       </c>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="12" t="n"/>
+      <c r="G8" s="10" t="n">
+        <v>71</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>1393.9</v>
+      </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
           <t>No</t>
@@ -1404,7 +1412,9 @@
       <c r="G13" s="7" t="n">
         <v>84</v>
       </c>
-      <c r="H13" s="13" t="n"/>
+      <c r="H13" s="13" t="n">
+        <v>1350.5</v>
+      </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
           <t>No</t>
@@ -1731,7 +1741,9 @@
       <c r="G20" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="H20" s="12" t="n"/>
+      <c r="H20" s="12" t="n">
+        <v>1357.1</v>
+      </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
           <t>No</t>
@@ -2196,8 +2208,12 @@
           <t>OFC</t>
         </is>
       </c>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="12" t="n"/>
+      <c r="G30" s="10" t="n">
+        <v>86</v>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>1343.8</v>
+      </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
           <t>No</t>
@@ -2289,7 +2305,9 @@
       <c r="G32" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="H32" s="12" t="n"/>
+      <c r="H32" s="12" t="n">
+        <v>1403.9</v>
+      </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
           <t>No</t>
@@ -2331,8 +2349,12 @@
           <t>AFC</t>
         </is>
       </c>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="13" t="n"/>
+      <c r="G33" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="H33" s="13" t="n">
+        <v>1430.6</v>
+      </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
           <t>No</t>
@@ -2515,8 +2537,12 @@
           <t>AFC</t>
         </is>
       </c>
-      <c r="G37" s="14" t="n"/>
-      <c r="H37" s="13" t="n"/>
+      <c r="G37" s="14" t="n">
+        <v>58</v>
+      </c>
+      <c r="H37" s="13" t="n">
+        <v>1437.3</v>
+      </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
           <t>No</t>
@@ -2749,7 +2775,9 @@
       <c r="G42" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="H42" s="12" t="n"/>
+      <c r="H42" s="12" t="n">
+        <v>1410.6</v>
+      </c>
       <c r="I42" s="10" t="inlineStr">
         <is>
           <t>No</t>
@@ -2885,8 +2913,12 @@
           <t>AFC</t>
         </is>
       </c>
-      <c r="G45" s="14" t="n"/>
-      <c r="H45" s="13" t="n"/>
+      <c r="G45" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="H45" s="13" t="n">
+        <v>1464</v>
+      </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
           <t>No</t>
@@ -3072,7 +3104,9 @@
       <c r="G49" s="7" t="n">
         <v>72</v>
       </c>
-      <c r="H49" s="13" t="n"/>
+      <c r="H49" s="13" t="n">
+        <v>1390.5</v>
+      </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
           <t>No</t>
@@ -3134,6 +3168,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="51"/>
     <row r="52" ht="15" customHeight="1" s="32">
       <c r="B52" s="33" t="inlineStr">
         <is>
@@ -11451,7 +11486,6 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="51"/>
     <row r="52" ht="15" customHeight="1" s="32">
       <c r="B52" s="33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Localia moderada para anfitriones en eliminatorias + hoja de sedes
- simulate.py: nuevo FACTOR_LOCALIA_KO=0.5; los anfitriones (MEX/USA/CAN) reciben una fraccion de la ventaja de localia en cada partido de eliminatoria (antes 100% neutral). Tuneable (0.0=neutral, 1.0=plena).
- Efecto: anfitriones pasan de ~13% a ~21% combinado (vs 53% con localia plena). USA/MEX ~8%. Con 0.3, Argentina sigue 1a.
- Excel: nueva hoja de referencia 'Sedes' (16 ciudades: pais, estadio, altitud) y columna 'Sede' agregada (vacia) en Fixture_Grupos y Eliminatorias para futuro mapeo partido->estadio.
- Docs: actualizada la decision de localia, parametros, snapshot y diccionario.
</commit_message>
<xml_diff>
--- a/Mundial_2026_fuente_datos.xlsx
+++ b/Mundial_2026_fuente_datos.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Fixture_Grupos" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Posiciones" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Eliminatorias" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Sedes" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -26,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -97,6 +98,9 @@
       <name val="Arial"/>
       <color rgb="FF000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -170,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -269,6 +273,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -829,6 +834,369 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>Sedes del Mundial 2026 (referencia: ciudad, país, estadio, altitud aprox. en m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>Ciudad</t>
+        </is>
+      </c>
+      <c r="B2" s="36" t="inlineStr">
+        <is>
+          <t>País</t>
+        </is>
+      </c>
+      <c r="C2" s="36" t="inlineStr">
+        <is>
+          <t>Estadio</t>
+        </is>
+      </c>
+      <c r="D2" s="36" t="inlineStr">
+        <is>
+          <t>Altitud (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ciudad de México</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Estadio Azteca</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Estadio Akron</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Estadio BBVA</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Canadá</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BMO Field</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Canadá</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BC Place</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nueva York/Nueva Jersey</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MetLife Stadium</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Dallas</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Los Ángeles</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Arrowhead Stadium</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bahía de San Francisco</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Levi's Stadium</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NRG Stadium</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Filadelfia</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lincoln Financial Field</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz Stadium</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Lumen Field</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hard Rock Stadium</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Gillette Stadium</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3168,7 +3536,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51"/>
     <row r="52" ht="15" customHeight="1" s="32">
       <c r="B52" s="33" t="inlineStr">
         <is>
@@ -11509,7 +11876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="32" min="1" max="1"/>
@@ -11576,6 +11943,11 @@
       <c r="J2" s="6" t="inlineStr">
         <is>
           <t>Pts B</t>
+        </is>
+      </c>
+      <c r="K2" s="36" t="inlineStr">
+        <is>
+          <t>Sede</t>
         </is>
       </c>
     </row>
@@ -17025,7 +17397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="32" min="1" max="1"/>
@@ -17079,6 +17451,11 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="H2" s="36" t="inlineStr">
+        <is>
+          <t>Sede</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="32">
       <c r="A3" s="7" t="inlineStr">

</xml_diff>